<commit_message>
7.1 activitiy + correct to 6.2 slides
</commit_message>
<xml_diff>
--- a/stat-3540-f26-schedule.xlsx
+++ b/stat-3540-f26-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8EB843-2D72-144E-B784-7B69382DC491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9009F3C6-770C-CD4A-931B-73DF23E82D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="84">
   <si>
     <t>week</t>
   </si>
@@ -282,6 +282,9 @@
   </si>
   <si>
     <t>https://docs.google.com/presentation/d/1dBzGEExrhUTM1T7zLMOr3MCZeZWTmTtMcCfUPAc3ogY/edit?usp=sharing</t>
+  </si>
+  <si>
+    <t>3-activities/instructions/07.1-activity-latin-squares.qmd</t>
   </si>
 </sst>
 </file>
@@ -1052,6 +1055,9 @@
         <v>80</v>
       </c>
       <c r="G15" s="7"/>
+      <c r="H15" s="7" t="s">
+        <v>83</v>
+      </c>
       <c r="I15" s="7"/>
     </row>
     <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>